<commit_message>
SCRUM-51: з task-board.xlsx прибрано SCRUM-64 (25 рядків)
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -639,28 +639,30 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-64</t>
+          <t>SCRUM-65</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>↳ Аудит розділів 1–2, 4, 6</t>
+          <t>↳ Аудит розділів 3, 5</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>ТА</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Коротка Ксенія</t>
+          <t>Тимчак Анастасія</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="4" t="n"/>
+      <c r="F5" s="3" t="n">
+        <v>4.5</v>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -668,7 +670,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Аркуш audit_korotka</t>
+          <t>Аркуш audit_tymchak</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -680,30 +682,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-65</t>
+          <t>SCRUM-66</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>↳ Аудит розділів 3, 5</t>
+          <t>↳ Аудит розділів 4, 5, 6</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>ТА</t>
+          <t>ІТ</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Тимчак Анастасія</t>
+          <t>Дрєпіна Анастасія</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="3" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="F6" s="4" t="n"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -711,7 +711,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Аркуш audit_tymchak</t>
+          <t>Аркуш audit_drepina</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -723,26 +723,26 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-66</t>
+          <t>SCRUM-67</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>↳ Аудит розділів 4, 5, 6</t>
+          <t>↳ Аудит розділів 1–2, 3</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>ІТ</t>
+          <t>СМ</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Дрєпіна Анастасія</t>
+          <t>Горбонос Олександра</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="3" t="inlineStr">
@@ -752,40 +752,42 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Аркуш audit_drepina</t>
+          <t>Аркуш audit_horbonos</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>СМ (рядки)</t>
+          <t>КТ (рядки)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-67</t>
+          <t>SCRUM-53</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>↳ Аудит розділів 1–2, 3</t>
+          <t>Зведення аркушів у єдиний реєстр дефектів</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>ТА</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Горбонос Олександра</t>
+          <t>Тимчак Анастасія</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -793,42 +795,40 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Аркуш audit_horbonos</t>
+          <t>Аркуш «Реєстр»</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>КТ (рядки)</t>
+          <t>СМ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-53</t>
+          <t>SCRUM-54</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Зведення аркушів у єдиний реєстр дефектів</t>
+          <t>«Адвокат замовника»: заперечення спірних рядків, аркуш «Спірні»</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>ТА</t>
+          <t>СМ</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Тимчак Анастасія</t>
+          <t>Горбонос Олександра</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="F9" s="4" t="n"/>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -836,38 +836,38 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Аркуш «Реєстр»</t>
+          <t>Аркуш «Спірні»</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>КТ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-54</t>
+          <t>SCRUM-55</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>«Адвокат замовника»: заперечення спірних рядків, аркуш «Спірні»</t>
+          <t>Модерація зведення і спірних, затвердження реєстру</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>КТ</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Горбонос Олександра</t>
+          <t>Коротка Ксенія</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="3" t="inlineStr">
@@ -877,48 +877,50 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Аркуш «Спірні»</t>
+          <t>Затверджений реєстр (аркуш «Реєстр»)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>СМ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-55</t>
+          <t>SCRUM-56</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Модерація зведення і спірних, затвердження реєстру</t>
+          <t>SRS 1.1 з журналом змін</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>ТА</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Коротка Ксенія</t>
+          <t>Тимчак Анастасія</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="4" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>готово</t>
+          <t>на рецензії</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Затверджений реєстр (аркуш «Реєстр»)</t>
+          <t>SRS-1.1.md (PR #28)</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -930,55 +932,51 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-56</t>
+          <t>SCRUM-57</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SRS 1.1 з журналом змін</t>
+          <t>План тестування продукту: 7 рівнів і типи (координація)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>ТА</t>
+          <t>ІТ</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Тимчак Анастасія</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>6</v>
-      </c>
+          <t>Дрєпіна Анастасія</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>на рецензії</t>
+          <t>готово</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>SRS-1.1.md (PR #28)</t>
+          <t>test-plan.md</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>СМ (чек-лист), КТ (пріоритети)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-57</t>
+          <t>SCRUM-68</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>План тестування продукту: 7 рівнів і типи (координація)</t>
+          <t>↳ Скелет плану: розділ 1, таблиця, 7 рівнів</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -991,8 +989,10 @@
           <t>Дрєпіна Анастасія</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="4" t="n"/>
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -1005,19 +1005,19 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>СМ (чек-лист), КТ (пріоритети)</t>
+          <t>СМ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-68</t>
+          <t>SCRUM-69</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>↳ Скелет плану: розділ 1, таблиця, 7 рівнів</t>
+          <t>↳ Типи 1–15 (функціональні та експлуатаційні)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1053,12 +1053,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-69</t>
+          <t>SCRUM-70</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>↳ Типи 1–15 (функціональні та експлуатаційні)</t>
+          <t>↳ Типи 16–24 (продуктивність) і незастосовні типи</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="3" t="inlineStr">
@@ -1094,12 +1094,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-70</t>
+          <t>SCRUM-71</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>↳ Типи 16–24 (продуктивність) і незастосовні типи</t>
+          <t>↳ Розділи 5–6 плану і прив'язка до ID з SRS 1.1</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>test-plan.md</t>
+          <t>test-plan.md (PR #27)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1135,26 +1135,26 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-71</t>
+          <t>SCRUM-58</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>↳ Розділи 5–6 плану і прив'язка до ID з SRS 1.1</t>
+          <t>Затвердження пріоритетів і застосовності типів у плані</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>ІТ</t>
+          <t>КТ</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Дрєпіна Анастасія</t>
+          <t>Коротка Ксенія</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>test-plan.md (PR #27)</t>
+          <t>Коментарі до плану (Jira SCRUM-58)</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1176,67 +1176,67 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-58</t>
+          <t>SCRUM-59</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Затвердження пріоритетів і застосовності типів у плані</t>
+          <t>Рецензування реєстру, SRS 1.1 і плану за офіційними чек-листами</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
+          <t>СМ</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Горбонос Олександра</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>в роботі</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Аркуш «Рецензування»</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
           <t>КТ</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Коротка Ксенія</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>готово</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Коментарі до плану (Jira SCRUM-58)</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>СМ</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-59</t>
+          <t>SCRUM-60</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Рецензування реєстру, SRS 1.1 і плану за офіційними чек-листами</t>
+          <t>Складання docs/sprint2/, README і перевірка DoD</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>КТ</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Горбонос Олександра</t>
+          <t>Коротка Ксенія</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="inlineStr">
@@ -1246,24 +1246,24 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Аркуш «Рецензування»</t>
+          <t>README.md</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>СМ</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-60</t>
+          <t>SCRUM-61</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Складання docs/sprint2/, README і перевірка DoD</t>
+          <t>Підготовка до презентації: демо (10 хв) і бліц</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1276,18 +1276,16 @@
           <t>Коротка Ксенія</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>в роботі</t>
+          <t>заплановано</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>Сценарій демо; бліц</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1299,12 +1297,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-61</t>
+          <t>SCRUM-72</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Підготовка до презентації: демо (10 хв) і бліц</t>
+          <t>↳ Сценарій демо і репетиція (10 хв)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1317,7 +1315,9 @@
           <t>Коротка Ксенія</t>
         </is>
       </c>
-      <c r="E21" s="3" t="n"/>
+      <c r="E21" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Сценарій демо; бліц</t>
+          <t>Сценарій демо</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1338,26 +1338,26 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-72</t>
+          <t>SCRUM-73</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>↳ Сценарій демо і репетиція (10 хв)</t>
+          <t>↳ Підготуватись пояснити реєстр і SRS 1.1 (три показові дефекти)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>ТА</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Коротка Ксенія</t>
+          <t>Тимчак Анастасія</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="inlineStr">
@@ -1367,34 +1367,34 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Сценарій демо</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>СМ</t>
+          <t>КТ</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-73</t>
+          <t>SCRUM-74</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>↳ Підготуватись пояснити реєстр і SRS 1.1 (три показові дефекти)</t>
+          <t>↳ Підготуватись пояснити план (пріоритети, два приклади Ціль/Опис)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ТА</t>
+          <t>ІТ</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Тимчак Анастасія</t>
+          <t>Дрєпіна Анастасія</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
@@ -1420,22 +1420,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-74</t>
+          <t>SCRUM-75</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>↳ Підготуватись пояснити план (пріоритети, два приклади Ціль/Опис)</t>
+          <t>↳ Спільна репетиція 12 бліц-питань і підготовка до ретро</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ІТ</t>
+          <t>СМ</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Дрєпіна Анастасія</t>
+          <t>Горбонос Олександра</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Шаблон протоколу ретро</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1461,12 +1461,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-75</t>
+          <t>SCRUM-62</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>↳ Спільна репетиція 12 бліц-питань і підготовка до ретро</t>
+          <t>Ретроспектива Start/Stop/Continue, протокол і peer-review</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Шаблон протоколу ретро</t>
+          <t>retro-sprint2.md</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SCRUM-62</t>
+          <t>SCRUM-63</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Ретроспектива Start/Stop/Continue, протокол і peer-review</t>
+          <t>(за бажанням) Виправлення зауважень спринта 1: BPMN-моделі і протокол рецензування</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1521,86 +1521,45 @@
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>заплановано</t>
+          <t>за бажанням (поза планом)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>retro-sprint2.md</t>
+          <t>docs/sprint1 (BPMN, протокол рецензування)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>КТ</t>
+          <t>ТА</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>SCRUM-63</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>(за бажанням) Виправлення зауважень спринта 1: BPMN-моделі і протокол рецензування</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>СМ</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Горбонос Олександра</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>за бажанням (поза планом)</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>docs/sprint1 (BPMN, протокол рецензування)</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>ТА</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="6">
-        <f>SUM(E2:E27)</f>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="6">
+        <f>SUM(E2:E26)</f>
         <v/>
       </c>
-      <c r="F28" s="6">
-        <f>SUM(F2:F27)</f>
+      <c r="F27" s="6">
+        <f>SUM(F2:F26)</f>
         <v/>
       </c>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1629,7 +1588,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1716,7 +1674,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Усі задачі й підзадачі спринта 2 (26 рядків). Підзадачі позначено «↳» і розташовано під батьківською задачею. Задачі спринта 1 (SCRUM-4, 18–21) не включено.</t>
+          <t>Задачі й підзадачі спринта 2 (25 рядків; SCRUM-64 не включено за рішенням СМ). Підзадачі позначено «↳» і розташовано під батьківською задачею. Задачі спринта 1 (SCRUM-4, 18–21) не включено.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCRUM-51: у task-board.xlsx внесено години СМ (SCRUM-51, 54, 59, 67)
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -580,7 +580,9 @@
       <c r="E3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="n"/>
+      <c r="F3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>в роботі</t>
@@ -785,7 +787,9 @@
       <c r="E8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -869,7 +873,9 @@
       <c r="E10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="4" t="n"/>
+      <c r="F10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -1238,7 +1244,9 @@
       <c r="E19" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="3" t="n"/>
+      <c r="F19" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
           <t>в роботі</t>
@@ -1710,7 +1718,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Години з worklog у Jira станом на 13.10.2026. Порожня клітинка — години в Jira не внесено. Жовтим виділено задачі «готово» без внесених годин.</t>
+          <t>Тимчак А. (SCRUM-53, 56, 65) — години з worklog Jira станом на 13.10.2026. Горбонос О. (SCRUM-51, 54, 59, 67) — внесено СМ у таблицю за обсягом оцінки; у Jira ці години ще не внесено. Порожня клітинка — годин немає (задача ще не виконувалась або години не внесено). Жовтим виділено задачі «готово» без годин.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCRUM-51: task-board.xlsx — додано години SCRUM-67 (3 год, Jira)
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -793,7 +793,9 @@
       <c r="E8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>готово</t>

</xml_diff>

<commit_message>
SCRUM-51: task-board.xlsx — додано години SCRUM-66 (2 год, Jira)
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -34,7 +34,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -79,9 +74,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -752,7 +744,9 @@
       <c r="E7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="4" t="n"/>
+      <c r="F7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -1573,25 +1567,25 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="6">
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="5">
         <f>SUM(E2:E26)</f>
         <v/>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="5">
         <f>SUM(F2:F26)</f>
         <v/>
       </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1639,7 +1633,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Продукт</t>
         </is>
@@ -1651,7 +1645,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Спринт</t>
         </is>
@@ -1663,7 +1657,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Дата експорту</t>
         </is>
@@ -1675,7 +1669,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Автор експорту</t>
         </is>
@@ -1687,7 +1681,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Джерело</t>
         </is>
@@ -1699,7 +1693,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Склад</t>
         </is>
@@ -1711,7 +1705,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Статуси</t>
         </is>
@@ -1723,7 +1717,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Оцінка</t>
         </is>
@@ -1735,7 +1729,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Факт</t>
         </is>
@@ -1747,7 +1741,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Доступ викладача</t>
         </is>

</xml_diff>

<commit_message>
SCRUM-62: task-board.xlsx — години SCRUM-73 (1 год, Jira)
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -34,7 +34,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -79,9 +74,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1432,7 +1424,9 @@
       <c r="E23" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="4" t="n"/>
+      <c r="F23" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>готово</t>
@@ -1577,25 +1571,25 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="6">
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="5">
         <f>SUM(E2:E26)</f>
         <v/>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="5">
         <f>SUM(F2:F26)</f>
         <v/>
       </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1643,7 +1637,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Продукт</t>
         </is>
@@ -1655,7 +1649,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Спринт</t>
         </is>
@@ -1667,7 +1661,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Дата експорту</t>
         </is>
@@ -1679,7 +1673,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Автор експорту</t>
         </is>
@@ -1691,7 +1685,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Джерело</t>
         </is>
@@ -1703,7 +1697,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Склад</t>
         </is>
@@ -1715,7 +1709,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Статуси</t>
         </is>
@@ -1727,7 +1721,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Оцінка</t>
         </is>
@@ -1739,7 +1733,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Факт</t>
         </is>
@@ -1751,7 +1745,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Доступ викладача</t>
         </is>

</xml_diff>